<commit_message>
Resultados de análisis problema3 (1M iteraciones)
</commit_message>
<xml_diff>
--- a/Nuevos DeepWins/Problem3_CheckerRotated/Res/Comparativa_12_Neuronas.xlsx
+++ b/Nuevos DeepWins/Problem3_CheckerRotated/Res/Comparativa_12_Neuronas.xlsx
@@ -581,35 +581,43 @@
         <v>0.1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.249384</v>
+        <v>0.241934</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1790731265</v>
+        <v>1790731213</v>
       </c>
       <c r="E2" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F2" t="n">
         <v>200000</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>0.547337</v>
+      </c>
       <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="inlineStr"/>
+        <v>0.48366</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.513532</v>
+      </c>
       <c r="J2" t="n">
-        <v>0.250385</v>
-      </c>
-      <c r="K2" t="inlineStr"/>
+        <v>0.25875</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.47644</v>
+      </c>
       <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="inlineStr"/>
+        <v>0.461929</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.469072</v>
+      </c>
       <c r="N2" t="n">
         <v>0.2</v>
       </c>
@@ -644,23 +652,23 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_0.txt</t>
+          <t>_2_12_1_1790731213_6.txt</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z2" t="n">
         <v>12</v>
       </c>
       <c r="AA2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -674,43 +682,35 @@
         <v>0.1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.242119</v>
+        <v>0.249518</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1790731213</v>
+        <v>1790731265</v>
       </c>
       <c r="E3" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F3" t="n">
         <v>200000</v>
       </c>
-      <c r="G3" t="n">
-        <v>0.531587</v>
-      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>0.45098</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.487977</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
-        <v>0.257878</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.471204</v>
-      </c>
+        <v>0.250158</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
-        <v>0.456853</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.463918</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
         <v>0.2</v>
       </c>
@@ -745,23 +745,23 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_17.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_13.txt</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z3" t="n">
         <v>12</v>
       </c>
       <c r="AA3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
@@ -775,35 +775,43 @@
         <v>0.1</v>
       </c>
       <c r="B4" t="n">
-        <v>0.249516</v>
+        <v>0.242071</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1790731265</v>
+        <v>1790731213</v>
       </c>
       <c r="E4" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F4" t="n">
         <v>200000</v>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>0.544207</v>
+      </c>
       <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="inlineStr"/>
+        <v>0.466667</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.502463</v>
+      </c>
       <c r="J4" t="n">
-        <v>0.250155</v>
-      </c>
-      <c r="K4" t="inlineStr"/>
+        <v>0.258707</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.468085</v>
+      </c>
       <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="inlineStr"/>
+        <v>0.446701</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.457143</v>
+      </c>
       <c r="N4" t="n">
         <v>0.2</v>
       </c>
@@ -838,23 +846,23 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_9.txt</t>
+          <t>_2_12_1_1790731213_2.txt</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z4" t="n">
         <v>12</v>
       </c>
       <c r="AA4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -868,7 +876,7 @@
         <v>0.1</v>
       </c>
       <c r="B5" t="n">
-        <v>0.241944</v>
+        <v>0.241989</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -885,25 +893,25 @@
         <v>200000</v>
       </c>
       <c r="G5" t="n">
-        <v>0.55</v>
+        <v>0.553159</v>
       </c>
       <c r="H5" t="n">
-        <v>0.47451</v>
+        <v>0.469281</v>
       </c>
       <c r="I5" t="n">
-        <v>0.509474</v>
+        <v>0.507779</v>
       </c>
       <c r="J5" t="n">
-        <v>0.25885</v>
+        <v>0.258842</v>
       </c>
       <c r="K5" t="n">
-        <v>0.47619</v>
+        <v>0.470899</v>
       </c>
       <c r="L5" t="n">
-        <v>0.456853</v>
+        <v>0.451777</v>
       </c>
       <c r="M5" t="n">
-        <v>0.466321</v>
+        <v>0.46114</v>
       </c>
       <c r="N5" t="n">
         <v>0.2</v>
@@ -939,7 +947,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_9.txt</t>
+          <t>_2_12_1_1790731213_16.txt</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -969,7 +977,7 @@
         <v>0.1</v>
       </c>
       <c r="B6" t="n">
-        <v>0.242176</v>
+        <v>0.242034</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -986,25 +994,25 @@
         <v>200000</v>
       </c>
       <c r="G6" t="n">
-        <v>0.534375</v>
+        <v>0.556231</v>
       </c>
       <c r="H6" t="n">
-        <v>0.447059</v>
+        <v>0.478431</v>
       </c>
       <c r="I6" t="n">
-        <v>0.486833</v>
+        <v>0.514406</v>
       </c>
       <c r="J6" t="n">
-        <v>0.257792</v>
+        <v>0.258783</v>
       </c>
       <c r="K6" t="n">
-        <v>0.484211</v>
+        <v>0.478495</v>
       </c>
       <c r="L6" t="n">
-        <v>0.467005</v>
+        <v>0.451777</v>
       </c>
       <c r="M6" t="n">
-        <v>0.475452</v>
+        <v>0.464752</v>
       </c>
       <c r="N6" t="n">
         <v>0.2</v>
@@ -1040,7 +1048,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_0.txt</t>
+          <t>_2_12_1_1790731213_4.txt</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1070,7 +1078,7 @@
         <v>0.1</v>
       </c>
       <c r="B7" t="n">
-        <v>0.249497</v>
+        <v>0.249517</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1092,7 +1100,7 @@
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="n">
-        <v>0.250177</v>
+        <v>0.250164</v>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
@@ -1133,7 +1141,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_12.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_6.txt</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -1163,7 +1171,7 @@
         <v>0.1</v>
       </c>
       <c r="B8" t="n">
-        <v>0.242074</v>
+        <v>0.242085</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1180,25 +1188,25 @@
         <v>200000</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5478</v>
+        <v>0.549853</v>
       </c>
       <c r="H8" t="n">
-        <v>0.471895</v>
+        <v>0.490196</v>
       </c>
       <c r="I8" t="n">
-        <v>0.507023</v>
+        <v>0.5183140000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>0.258788</v>
+        <v>0.259033</v>
       </c>
       <c r="K8" t="n">
-        <v>0.471204</v>
+        <v>0.466667</v>
       </c>
       <c r="L8" t="n">
-        <v>0.456853</v>
+        <v>0.461929</v>
       </c>
       <c r="M8" t="n">
-        <v>0.463918</v>
+        <v>0.464286</v>
       </c>
       <c r="N8" t="n">
         <v>0.2</v>
@@ -1234,7 +1242,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_18.txt</t>
+          <t>_2_12_1_1790731213_8.txt</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
@@ -1264,7 +1272,7 @@
         <v>0.1</v>
       </c>
       <c r="B9" t="n">
-        <v>0.249512</v>
+        <v>0.249384</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1286,7 +1294,7 @@
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
-        <v>0.250164</v>
+        <v>0.250385</v>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
@@ -1327,7 +1335,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_18.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_0.txt</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -1357,43 +1365,35 @@
         <v>0.1</v>
       </c>
       <c r="B10" t="n">
-        <v>0.241969</v>
+        <v>0.249516</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1790731213</v>
+        <v>1790731265</v>
       </c>
       <c r="E10" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F10" t="n">
         <v>200000</v>
       </c>
-      <c r="G10" t="n">
-        <v>0.543544</v>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>0.473203</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0.5059399999999999</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
-        <v>0.258952</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.466321</v>
-      </c>
+        <v>0.250155</v>
+      </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
-        <v>0.456853</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.461538</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
         <v>0.2</v>
       </c>
@@ -1428,23 +1428,23 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_5.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_9.txt</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z10" t="n">
         <v>12</v>
       </c>
       <c r="AA10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
@@ -1458,43 +1458,35 @@
         <v>0.1</v>
       </c>
       <c r="B11" t="n">
-        <v>0.242215</v>
+        <v>0.249517</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1790731213</v>
+        <v>1790731265</v>
       </c>
       <c r="E11" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F11" t="n">
         <v>200000</v>
       </c>
-      <c r="G11" t="n">
-        <v>0.535494</v>
-      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>0.453595</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0.491154</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
-        <v>0.258577</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0.467005</v>
-      </c>
+        <v>0.250154</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>0.467005</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0.467005</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
         <v>0.2</v>
       </c>
@@ -1529,23 +1521,23 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_12.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_2.txt</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z11" t="n">
         <v>12</v>
       </c>
       <c r="AA11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
@@ -1559,7 +1551,7 @@
         <v>0.1</v>
       </c>
       <c r="B12" t="n">
-        <v>0.242034</v>
+        <v>0.242239</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1576,25 +1568,25 @@
         <v>200000</v>
       </c>
       <c r="G12" t="n">
-        <v>0.556231</v>
+        <v>0.544049</v>
       </c>
       <c r="H12" t="n">
-        <v>0.478431</v>
+        <v>0.460131</v>
       </c>
       <c r="I12" t="n">
-        <v>0.514406</v>
+        <v>0.498584</v>
       </c>
       <c r="J12" t="n">
-        <v>0.258783</v>
+        <v>0.25872</v>
       </c>
       <c r="K12" t="n">
-        <v>0.478495</v>
+        <v>0.46114</v>
       </c>
       <c r="L12" t="n">
         <v>0.451777</v>
       </c>
       <c r="M12" t="n">
-        <v>0.464752</v>
+        <v>0.45641</v>
       </c>
       <c r="N12" t="n">
         <v>0.2</v>
@@ -1630,7 +1622,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_4.txt</t>
+          <t>_2_12_1_1790731213_19.txt</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
@@ -1660,43 +1652,35 @@
         <v>0.1</v>
       </c>
       <c r="B13" t="n">
-        <v>0.241862</v>
+        <v>0.249506</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1790731213</v>
+        <v>1790731265</v>
       </c>
       <c r="E13" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F13" t="n">
         <v>200000</v>
       </c>
-      <c r="G13" t="n">
-        <v>0.546256</v>
-      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>0.486275</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0.514523</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="n">
-        <v>0.258506</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0.466321</v>
-      </c>
+        <v>0.250125</v>
+      </c>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
-        <v>0.456853</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0.461538</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
         <v>0.2</v>
       </c>
@@ -1731,23 +1715,23 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_13.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_17.txt</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z13" t="n">
         <v>12</v>
       </c>
       <c r="AA13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
@@ -1761,35 +1745,43 @@
         <v>0.1</v>
       </c>
       <c r="B14" t="n">
-        <v>0.249517</v>
+        <v>0.242204</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1790731265</v>
+        <v>1790731213</v>
       </c>
       <c r="E14" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F14" t="n">
         <v>200000</v>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="n">
+        <v>0.5387</v>
+      </c>
       <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="inlineStr"/>
+        <v>0.454902</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.493267</v>
+      </c>
       <c r="J14" t="n">
-        <v>0.250164</v>
-      </c>
-      <c r="K14" t="inlineStr"/>
+        <v>0.257921</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.478495</v>
+      </c>
       <c r="L14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" t="inlineStr"/>
+        <v>0.451777</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.464752</v>
+      </c>
       <c r="N14" t="n">
         <v>0.2</v>
       </c>
@@ -1824,23 +1816,23 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_6.txt</t>
+          <t>_2_12_1_1790731213_1.txt</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z14" t="n">
         <v>12</v>
       </c>
       <c r="AA14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
@@ -1854,7 +1846,7 @@
         <v>0.1</v>
       </c>
       <c r="B15" t="n">
-        <v>0.249345</v>
+        <v>0.249422</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1876,7 +1868,7 @@
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="n">
-        <v>0.2505</v>
+        <v>0.25031</v>
       </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
@@ -1917,7 +1909,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_8.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_15.txt</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
@@ -1947,35 +1939,43 @@
         <v>0.1</v>
       </c>
       <c r="B16" t="n">
-        <v>0.249499</v>
+        <v>0.242074</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1790731265</v>
+        <v>1790731213</v>
       </c>
       <c r="E16" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F16" t="n">
         <v>200000</v>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="n">
+        <v>0.5478</v>
+      </c>
       <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="inlineStr"/>
+        <v>0.471895</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.507023</v>
+      </c>
       <c r="J16" t="n">
-        <v>0.250236</v>
-      </c>
-      <c r="K16" t="inlineStr"/>
+        <v>0.258788</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.471204</v>
+      </c>
       <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="inlineStr"/>
+        <v>0.456853</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.463918</v>
+      </c>
       <c r="N16" t="n">
         <v>0.2</v>
       </c>
@@ -2010,23 +2010,23 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_7.txt</t>
+          <t>_2_12_1_1790731213_18.txt</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z16" t="n">
         <v>12</v>
       </c>
       <c r="AA16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
@@ -2040,7 +2040,7 @@
         <v>0.1</v>
       </c>
       <c r="B17" t="n">
-        <v>0.249506</v>
+        <v>0.249512</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="n">
-        <v>0.250125</v>
+        <v>0.250164</v>
       </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_17.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_18.txt</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
@@ -2133,7 +2133,7 @@
         <v>0.1</v>
       </c>
       <c r="B18" t="n">
-        <v>0.249422</v>
+        <v>0.249387</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2155,7 +2155,7 @@
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="n">
-        <v>0.25031</v>
+        <v>0.250371</v>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_15.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_4.txt</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -2327,43 +2327,35 @@
         <v>0.1</v>
       </c>
       <c r="B20" t="n">
-        <v>0.242149</v>
+        <v>0.249497</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1790731213</v>
+        <v>1790731265</v>
       </c>
       <c r="E20" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F20" t="n">
         <v>200000</v>
       </c>
-      <c r="G20" t="n">
-        <v>0.540909</v>
-      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>0.466667</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0.501053</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
       <c r="J20" t="n">
-        <v>0.257625</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0.474227</v>
-      </c>
+        <v>0.250177</v>
+      </c>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="n">
-        <v>0.467005</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0.470588</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="n">
         <v>0.2</v>
       </c>
@@ -2398,23 +2390,23 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_10.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_12.txt</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z20" t="n">
         <v>12</v>
       </c>
       <c r="AA20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -2428,7 +2420,7 @@
         <v>0.1</v>
       </c>
       <c r="B21" t="n">
-        <v>0.242204</v>
+        <v>0.242059</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2445,25 +2437,25 @@
         <v>200000</v>
       </c>
       <c r="G21" t="n">
-        <v>0.5387</v>
+        <v>0.54977</v>
       </c>
       <c r="H21" t="n">
-        <v>0.454902</v>
+        <v>0.469281</v>
       </c>
       <c r="I21" t="n">
-        <v>0.493267</v>
+        <v>0.506347</v>
       </c>
       <c r="J21" t="n">
-        <v>0.257921</v>
+        <v>0.258829</v>
       </c>
       <c r="K21" t="n">
-        <v>0.478495</v>
+        <v>0.478723</v>
       </c>
       <c r="L21" t="n">
-        <v>0.451777</v>
+        <v>0.456853</v>
       </c>
       <c r="M21" t="n">
-        <v>0.464752</v>
+        <v>0.467532</v>
       </c>
       <c r="N21" t="n">
         <v>0.2</v>
@@ -2499,7 +2491,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_1.txt</t>
+          <t>_2_12_1_1790731213_3.txt</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
@@ -2529,43 +2521,35 @@
         <v>0.1</v>
       </c>
       <c r="B22" t="n">
-        <v>0.242239</v>
+        <v>0.249518</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1790731213</v>
+        <v>1790731265</v>
       </c>
       <c r="E22" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F22" t="n">
         <v>200000</v>
       </c>
-      <c r="G22" t="n">
-        <v>0.544049</v>
-      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>0.460131</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0.498584</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr"/>
       <c r="J22" t="n">
-        <v>0.25872</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0.46114</v>
-      </c>
+        <v>0.25015</v>
+      </c>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="n">
-        <v>0.451777</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0.45641</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
         <v>0.2</v>
       </c>
@@ -2600,23 +2584,23 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_19.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_3.txt</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z22" t="n">
         <v>12</v>
       </c>
       <c r="AA22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC22" t="inlineStr">
@@ -2630,7 +2614,7 @@
         <v>0.1</v>
       </c>
       <c r="B23" t="n">
-        <v>0.248897</v>
+        <v>0.249499</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2646,27 +2630,19 @@
       <c r="F23" t="n">
         <v>200000</v>
       </c>
-      <c r="G23" t="n">
-        <v>0.563422</v>
-      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>0.249673</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0.346015</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="n">
-        <v>0.251643</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0.431373</v>
-      </c>
+        <v>0.250236</v>
+      </c>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="n">
-        <v>0.22335</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0.294314</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="n">
         <v>0.2</v>
       </c>
@@ -2701,7 +2677,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_19.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_7.txt</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
@@ -2731,43 +2707,35 @@
         <v>0.1</v>
       </c>
       <c r="B24" t="n">
-        <v>0.242071</v>
+        <v>0.249345</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1790731213</v>
+        <v>1790731265</v>
       </c>
       <c r="E24" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F24" t="n">
         <v>200000</v>
       </c>
-      <c r="G24" t="n">
-        <v>0.544207</v>
-      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>0.466667</v>
-      </c>
-      <c r="I24" t="n">
-        <v>0.502463</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="n">
-        <v>0.258707</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0.468085</v>
-      </c>
+        <v>0.2505</v>
+      </c>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="n">
-        <v>0.446701</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0.457143</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M24" t="inlineStr"/>
       <c r="N24" t="n">
         <v>0.2</v>
       </c>
@@ -2802,23 +2770,23 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_2.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_8.txt</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z24" t="n">
         <v>12</v>
       </c>
       <c r="AA24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC24" t="inlineStr">
@@ -2832,35 +2800,43 @@
         <v>0.1</v>
       </c>
       <c r="B25" t="n">
-        <v>0.249077</v>
+        <v>0.242149</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>1790731265</v>
+        <v>1790731213</v>
       </c>
       <c r="E25" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F25" t="n">
         <v>200000</v>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="n">
+        <v>0.540909</v>
+      </c>
       <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="inlineStr"/>
+        <v>0.466667</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.501053</v>
+      </c>
       <c r="J25" t="n">
-        <v>0.251382</v>
-      </c>
-      <c r="K25" t="inlineStr"/>
+        <v>0.257625</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.474227</v>
+      </c>
       <c r="L25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" t="inlineStr"/>
+        <v>0.467005</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.470588</v>
+      </c>
       <c r="N25" t="n">
         <v>0.2</v>
       </c>
@@ -2895,23 +2871,23 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_14.txt</t>
+          <t>_2_12_1_1790731213_10.txt</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z25" t="n">
         <v>12</v>
       </c>
       <c r="AA25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC25" t="inlineStr">
@@ -2925,42 +2901,42 @@
         <v>0.1</v>
       </c>
       <c r="B26" t="n">
-        <v>0.248965</v>
+        <v>0.242194</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1790731265</v>
+        <v>1790731213</v>
       </c>
       <c r="E26" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F26" t="n">
         <v>200000</v>
       </c>
       <c r="G26" t="n">
-        <v>0.517483</v>
+        <v>0.540193</v>
       </c>
       <c r="H26" t="n">
-        <v>0.290196</v>
+        <v>0.439216</v>
       </c>
       <c r="I26" t="n">
-        <v>0.371859</v>
+        <v>0.484499</v>
       </c>
       <c r="J26" t="n">
-        <v>0.252038</v>
+        <v>0.258459</v>
       </c>
       <c r="K26" t="n">
-        <v>0.444444</v>
+        <v>0.494505</v>
       </c>
       <c r="L26" t="n">
-        <v>0.284264</v>
+        <v>0.456853</v>
       </c>
       <c r="M26" t="n">
-        <v>0.346749</v>
+        <v>0.474934</v>
       </c>
       <c r="N26" t="n">
         <v>0.2</v>
@@ -2996,23 +2972,23 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_16.txt</t>
+          <t>_2_12_1_1790731213_11.txt</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z26" t="n">
         <v>12</v>
       </c>
       <c r="AA26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC26" t="inlineStr">
@@ -3026,7 +3002,7 @@
         <v>0.1</v>
       </c>
       <c r="B27" t="n">
-        <v>0.249523</v>
+        <v>0.248965</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -3042,19 +3018,27 @@
       <c r="F27" t="n">
         <v>200000</v>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="n">
+        <v>0.517483</v>
+      </c>
       <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" t="inlineStr"/>
+        <v>0.290196</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.371859</v>
+      </c>
       <c r="J27" t="n">
-        <v>0.250158</v>
-      </c>
-      <c r="K27" t="inlineStr"/>
+        <v>0.252038</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.444444</v>
+      </c>
       <c r="L27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" t="inlineStr"/>
+        <v>0.284264</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0.346749</v>
+      </c>
       <c r="N27" t="n">
         <v>0.2</v>
       </c>
@@ -3089,7 +3073,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_10.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_16.txt</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
@@ -3119,7 +3103,7 @@
         <v>0.1</v>
       </c>
       <c r="B28" t="n">
-        <v>0.249387</v>
+        <v>0.249521</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -3141,7 +3125,7 @@
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="n">
-        <v>0.250371</v>
+        <v>0.250151</v>
       </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
@@ -3182,7 +3166,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_4.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_11.txt</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
@@ -3212,7 +3196,7 @@
         <v>0.1</v>
       </c>
       <c r="B29" t="n">
-        <v>0.249518</v>
+        <v>0.249077</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3234,7 +3218,7 @@
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="n">
-        <v>0.25015</v>
+        <v>0.251382</v>
       </c>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="n">
@@ -3275,7 +3259,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_3.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_14.txt</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
@@ -3305,43 +3289,35 @@
         <v>0.1</v>
       </c>
       <c r="B30" t="n">
-        <v>0.241871</v>
+        <v>0.249496</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1790731213</v>
+        <v>1790731265</v>
       </c>
       <c r="E30" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F30" t="n">
         <v>200000</v>
       </c>
-      <c r="G30" t="n">
-        <v>0.554033</v>
-      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>0.475817</v>
-      </c>
-      <c r="I30" t="n">
-        <v>0.511955</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr"/>
       <c r="J30" t="n">
-        <v>0.258919</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0.489691</v>
-      </c>
+        <v>0.250197</v>
+      </c>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="n">
-        <v>0.482233</v>
-      </c>
-      <c r="M30" t="n">
-        <v>0.485934</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M30" t="inlineStr"/>
       <c r="N30" t="n">
         <v>0.2</v>
       </c>
@@ -3376,23 +3352,23 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_7.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_1.txt</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z30" t="n">
         <v>12</v>
       </c>
       <c r="AA30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC30" t="inlineStr">
@@ -3406,42 +3382,42 @@
         <v>0.1</v>
       </c>
       <c r="B31" t="n">
-        <v>0.242093</v>
+        <v>0.248897</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1790731213</v>
+        <v>1790731265</v>
       </c>
       <c r="E31" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F31" t="n">
         <v>200000</v>
       </c>
       <c r="G31" t="n">
-        <v>0.531202</v>
+        <v>0.563422</v>
       </c>
       <c r="H31" t="n">
-        <v>0.456209</v>
+        <v>0.249673</v>
       </c>
       <c r="I31" t="n">
-        <v>0.490858</v>
+        <v>0.346015</v>
       </c>
       <c r="J31" t="n">
-        <v>0.25778</v>
+        <v>0.251643</v>
       </c>
       <c r="K31" t="n">
-        <v>0.479381</v>
+        <v>0.431373</v>
       </c>
       <c r="L31" t="n">
-        <v>0.472081</v>
+        <v>0.22335</v>
       </c>
       <c r="M31" t="n">
-        <v>0.475703</v>
+        <v>0.294314</v>
       </c>
       <c r="N31" t="n">
         <v>0.2</v>
@@ -3477,23 +3453,23 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_14.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_19.txt</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z31" t="n">
         <v>12</v>
       </c>
       <c r="AA31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
@@ -3507,43 +3483,35 @@
         <v>0.1</v>
       </c>
       <c r="B32" t="n">
-        <v>0.241934</v>
+        <v>0.24945</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1790731213</v>
+        <v>1790731265</v>
       </c>
       <c r="E32" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F32" t="n">
         <v>200000</v>
       </c>
-      <c r="G32" t="n">
-        <v>0.547337</v>
-      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>0.48366</v>
-      </c>
-      <c r="I32" t="n">
-        <v>0.513532</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
       <c r="J32" t="n">
-        <v>0.25875</v>
-      </c>
-      <c r="K32" t="n">
-        <v>0.47644</v>
-      </c>
+        <v>0.250291</v>
+      </c>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="n">
-        <v>0.461929</v>
-      </c>
-      <c r="M32" t="n">
-        <v>0.469072</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M32" t="inlineStr"/>
       <c r="N32" t="n">
         <v>0.2</v>
       </c>
@@ -3578,23 +3546,23 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_6.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_5.txt</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z32" t="n">
         <v>12</v>
       </c>
       <c r="AA32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
@@ -3608,7 +3576,7 @@
         <v>0.1</v>
       </c>
       <c r="B33" t="n">
-        <v>0.241989</v>
+        <v>0.241944</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3625,25 +3593,25 @@
         <v>200000</v>
       </c>
       <c r="G33" t="n">
-        <v>0.553159</v>
+        <v>0.55</v>
       </c>
       <c r="H33" t="n">
-        <v>0.469281</v>
+        <v>0.47451</v>
       </c>
       <c r="I33" t="n">
-        <v>0.507779</v>
+        <v>0.509474</v>
       </c>
       <c r="J33" t="n">
-        <v>0.258842</v>
+        <v>0.25885</v>
       </c>
       <c r="K33" t="n">
-        <v>0.470899</v>
+        <v>0.47619</v>
       </c>
       <c r="L33" t="n">
-        <v>0.451777</v>
+        <v>0.456853</v>
       </c>
       <c r="M33" t="n">
-        <v>0.46114</v>
+        <v>0.466321</v>
       </c>
       <c r="N33" t="n">
         <v>0.2</v>
@@ -3679,7 +3647,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_16.txt</t>
+          <t>_2_12_1_1790731213_9.txt</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
@@ -3709,35 +3677,43 @@
         <v>0.1</v>
       </c>
       <c r="B34" t="n">
-        <v>0.249496</v>
+        <v>0.241862</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1790731265</v>
+        <v>1790731213</v>
       </c>
       <c r="E34" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F34" t="n">
         <v>200000</v>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="G34" t="n">
+        <v>0.546256</v>
+      </c>
       <c r="H34" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" t="inlineStr"/>
+        <v>0.486275</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.514523</v>
+      </c>
       <c r="J34" t="n">
-        <v>0.250197</v>
-      </c>
-      <c r="K34" t="inlineStr"/>
+        <v>0.258506</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0.466321</v>
+      </c>
       <c r="L34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M34" t="inlineStr"/>
+        <v>0.456853</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0.461538</v>
+      </c>
       <c r="N34" t="n">
         <v>0.2</v>
       </c>
@@ -3772,23 +3748,23 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_1.txt</t>
+          <t>_2_12_1_1790731213_13.txt</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z34" t="n">
         <v>12</v>
       </c>
       <c r="AA34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC34" t="inlineStr">
@@ -3802,35 +3778,43 @@
         <v>0.1</v>
       </c>
       <c r="B35" t="n">
-        <v>0.249521</v>
+        <v>0.242119</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1790731265</v>
+        <v>1790731213</v>
       </c>
       <c r="E35" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F35" t="n">
         <v>200000</v>
       </c>
-      <c r="G35" t="inlineStr"/>
+      <c r="G35" t="n">
+        <v>0.531587</v>
+      </c>
       <c r="H35" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" t="inlineStr"/>
+        <v>0.45098</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.487977</v>
+      </c>
       <c r="J35" t="n">
-        <v>0.250151</v>
-      </c>
-      <c r="K35" t="inlineStr"/>
+        <v>0.257878</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.471204</v>
+      </c>
       <c r="L35" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" t="inlineStr"/>
+        <v>0.456853</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0.463918</v>
+      </c>
       <c r="N35" t="n">
         <v>0.2</v>
       </c>
@@ -3865,23 +3849,23 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_11.txt</t>
+          <t>_2_12_1_1790731213_17.txt</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z35" t="n">
         <v>12</v>
       </c>
       <c r="AA35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC35" t="inlineStr">
@@ -3895,35 +3879,43 @@
         <v>0.1</v>
       </c>
       <c r="B36" t="n">
-        <v>0.249517</v>
+        <v>0.242215</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1790731265</v>
+        <v>1790731213</v>
       </c>
       <c r="E36" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F36" t="n">
         <v>200000</v>
       </c>
-      <c r="G36" t="inlineStr"/>
+      <c r="G36" t="n">
+        <v>0.535494</v>
+      </c>
       <c r="H36" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" t="inlineStr"/>
+        <v>0.453595</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.491154</v>
+      </c>
       <c r="J36" t="n">
-        <v>0.250154</v>
-      </c>
-      <c r="K36" t="inlineStr"/>
+        <v>0.258577</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0.467005</v>
+      </c>
       <c r="L36" t="n">
-        <v>0</v>
-      </c>
-      <c r="M36" t="inlineStr"/>
+        <v>0.467005</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0.467005</v>
+      </c>
       <c r="N36" t="n">
         <v>0.2</v>
       </c>
@@ -3958,23 +3950,23 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_2.txt</t>
+          <t>_2_12_1_1790731213_12.txt</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z36" t="n">
         <v>12</v>
       </c>
       <c r="AA36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC36" t="inlineStr">
@@ -3988,7 +3980,7 @@
         <v>0.1</v>
       </c>
       <c r="B37" t="n">
-        <v>0.242085</v>
+        <v>0.241969</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -4005,25 +3997,25 @@
         <v>200000</v>
       </c>
       <c r="G37" t="n">
-        <v>0.549853</v>
+        <v>0.543544</v>
       </c>
       <c r="H37" t="n">
-        <v>0.490196</v>
+        <v>0.473203</v>
       </c>
       <c r="I37" t="n">
-        <v>0.5183140000000001</v>
+        <v>0.5059399999999999</v>
       </c>
       <c r="J37" t="n">
-        <v>0.259033</v>
+        <v>0.258952</v>
       </c>
       <c r="K37" t="n">
-        <v>0.466667</v>
+        <v>0.466321</v>
       </c>
       <c r="L37" t="n">
-        <v>0.461929</v>
+        <v>0.456853</v>
       </c>
       <c r="M37" t="n">
-        <v>0.464286</v>
+        <v>0.461538</v>
       </c>
       <c r="N37" t="n">
         <v>0.2</v>
@@ -4059,7 +4051,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_8.txt</t>
+          <t>_2_12_1_1790731213_5.txt</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
@@ -4089,35 +4081,43 @@
         <v>0.1</v>
       </c>
       <c r="B38" t="n">
-        <v>0.249518</v>
+        <v>0.241871</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1790731265</v>
+        <v>1790731213</v>
       </c>
       <c r="E38" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F38" t="n">
         <v>200000</v>
       </c>
-      <c r="G38" t="inlineStr"/>
+      <c r="G38" t="n">
+        <v>0.554033</v>
+      </c>
       <c r="H38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" t="inlineStr"/>
+        <v>0.475817</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.511955</v>
+      </c>
       <c r="J38" t="n">
-        <v>0.250158</v>
-      </c>
-      <c r="K38" t="inlineStr"/>
+        <v>0.258919</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.489691</v>
+      </c>
       <c r="L38" t="n">
-        <v>0</v>
-      </c>
-      <c r="M38" t="inlineStr"/>
+        <v>0.482233</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0.485934</v>
+      </c>
       <c r="N38" t="n">
         <v>0.2</v>
       </c>
@@ -4152,23 +4152,23 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_13.txt</t>
+          <t>_2_12_1_1790731213_7.txt</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z38" t="n">
         <v>12</v>
       </c>
       <c r="AA38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC38" t="inlineStr">
@@ -4182,35 +4182,43 @@
         <v>0.1</v>
       </c>
       <c r="B39" t="n">
-        <v>0.24945</v>
+        <v>0.242176</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1790731265</v>
+        <v>1790731213</v>
       </c>
       <c r="E39" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F39" t="n">
         <v>200000</v>
       </c>
-      <c r="G39" t="inlineStr"/>
+      <c r="G39" t="n">
+        <v>0.534375</v>
+      </c>
       <c r="H39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" t="inlineStr"/>
+        <v>0.447059</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.486833</v>
+      </c>
       <c r="J39" t="n">
-        <v>0.250291</v>
-      </c>
-      <c r="K39" t="inlineStr"/>
+        <v>0.257792</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.484211</v>
+      </c>
       <c r="L39" t="n">
-        <v>0</v>
-      </c>
-      <c r="M39" t="inlineStr"/>
+        <v>0.467005</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0.475452</v>
+      </c>
       <c r="N39" t="n">
         <v>0.2</v>
       </c>
@@ -4245,23 +4253,23 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790731265_5.txt</t>
+          <t>_2_12_1_1790731213_0.txt</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z39" t="n">
         <v>12</v>
       </c>
       <c r="AA39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC39" t="inlineStr">
@@ -4275,7 +4283,7 @@
         <v>0.1</v>
       </c>
       <c r="B40" t="n">
-        <v>0.242194</v>
+        <v>0.242093</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -4292,25 +4300,25 @@
         <v>200000</v>
       </c>
       <c r="G40" t="n">
-        <v>0.540193</v>
+        <v>0.531202</v>
       </c>
       <c r="H40" t="n">
-        <v>0.439216</v>
+        <v>0.456209</v>
       </c>
       <c r="I40" t="n">
-        <v>0.484499</v>
+        <v>0.490858</v>
       </c>
       <c r="J40" t="n">
-        <v>0.258459</v>
+        <v>0.25778</v>
       </c>
       <c r="K40" t="n">
-        <v>0.494505</v>
+        <v>0.479381</v>
       </c>
       <c r="L40" t="n">
-        <v>0.456853</v>
+        <v>0.472081</v>
       </c>
       <c r="M40" t="n">
-        <v>0.474934</v>
+        <v>0.475703</v>
       </c>
       <c r="N40" t="n">
         <v>0.2</v>
@@ -4346,7 +4354,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_11.txt</t>
+          <t>_2_12_1_1790731213_14.txt</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
@@ -4376,43 +4384,35 @@
         <v>0.1</v>
       </c>
       <c r="B41" t="n">
-        <v>0.242059</v>
+        <v>0.249523</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1790731213</v>
+        <v>1790731265</v>
       </c>
       <c r="E41" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F41" t="n">
         <v>200000</v>
       </c>
-      <c r="G41" t="n">
-        <v>0.54977</v>
-      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>0.469281</v>
-      </c>
-      <c r="I41" t="n">
-        <v>0.506347</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I41" t="inlineStr"/>
       <c r="J41" t="n">
-        <v>0.258829</v>
-      </c>
-      <c r="K41" t="n">
-        <v>0.478723</v>
-      </c>
+        <v>0.250158</v>
+      </c>
+      <c r="K41" t="inlineStr"/>
       <c r="L41" t="n">
-        <v>0.456853</v>
-      </c>
-      <c r="M41" t="n">
-        <v>0.467532</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M41" t="inlineStr"/>
       <c r="N41" t="n">
         <v>0.2</v>
       </c>
@@ -4447,23 +4447,23 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>_2_12_1_1790731213_3.txt</t>
+          <t>_2_3_3_3_3_1_1790731265_10.txt</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z41" t="n">
         <v>12</v>
       </c>
       <c r="AA41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC41" t="inlineStr">
@@ -4538,7 +4538,7 @@
         <v>0.4669734</v>
       </c>
       <c r="C2" t="n">
-        <v>0.006983395361781219</v>
+        <v>0.006983395361781225</v>
       </c>
       <c r="D2" t="n">
         <v>0.485934</v>
@@ -4566,7 +4566,7 @@
         <v>0.3205315</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0370771440715166</v>
+        <v>0.03707714407151657</v>
       </c>
       <c r="D3" t="n">
         <v>0.346749</v>

</xml_diff>